<commit_message>
Leads: 2026-10-09 05:41 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-09.xlsx
+++ b/output/leads_2026-10-09.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -524,7 +524,6 @@
           <t>https://www.riosroofinglaredo.com/</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>oriosroofing@gmail.com</t>
@@ -554,6 +553,66 @@
         </is>
       </c>
       <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>The Plumber: Plumbing Services in Palmdale, CA</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>theplumberav.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://www.theplumberav.com/plumber-palmdale-ca</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Antelope Valley</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>iamtheplumber1@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>661-722-6039</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Palmdale CA</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>plumber Palmdale CA</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-09 05:45 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-09.xlsx
+++ b/output/leads_2026-10-09.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -618,6 +618,62 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Baker Plumbing</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>bakerplumbingfl.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://www.bakerplumbingfl.com/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Area Latest</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>bakerplumbingfl@gmail.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Cape Coral FL</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>76</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>plumber Cape Coral FL</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-09 05:48 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-09.xlsx
+++ b/output/leads_2026-10-09.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -649,7 +649,6 @@
           <t>bakerplumbingfl@gmail.com</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>Cape Coral FL</t>
@@ -669,6 +668,67 @@
         </is>
       </c>
       <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Air Conditioning Repair and Service
+Air Conditioning Cleaning, Tune up and Stea</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>brooklynhvacsolutions.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://brooklynhvacsolutions.com/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>info@brooklynhvacsolutions.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(631) 533-0542</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>90</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>air conditioning repair Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-09 05:50 UTC (cycle 14)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-09.xlsx
+++ b/output/leads_2026-10-09.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -734,6 +734,66 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Metal Roof Company | Cleveland, OH | Apex Exterior Pros LLC</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>apexextplus.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.apexextplus.com/metal-roof-installation-northeast-ohio</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Apex Exterior</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>apex.pro.gus@gmail.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(330) 979-1795</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Cleveland OH</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>90</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Cleveland OH</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-09 15:14 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-09.xlsx
+++ b/output/leads_2026-10-09.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -794,6 +794,62 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Got Your Six Heating &amp; Cooling in Brownsville</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>gotyoursixheatingcooling.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://gotyoursixheatingcooling.com/locations/brownsville-tx/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>info@gotyoursixheatingcooling.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>(888) 977-3905</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Brownsville TX</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>90</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>heating and cooling company Brownsville TX</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-09 15:26 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-09.xlsx
+++ b/output/leads_2026-10-09.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -815,7 +815,6 @@
           <t>https://gotyoursixheatingcooling.com/locations/brownsville-tx/</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>info@gotyoursixheatingcooling.com</t>
@@ -845,6 +844,66 @@
         </is>
       </c>
       <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>National Furnace &amp; Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>nationalfurnace.net</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://nationalfurnace.net/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Serving Lincoln</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>nationalfurnace@gmail.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>402-436-3492</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Lincoln NE</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>100</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>furnace repair Lincoln NE</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-09 15:27 UTC (cycle 14)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-09.xlsx
+++ b/output/leads_2026-10-09.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -909,6 +909,122 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Global Roofing and Construction</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>globalroofer.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://globalroofer.com/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Central Ka</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>info@globalroofer.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(316) 469-5023</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Wichita KS</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>80</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>roofing contractor Wichita KS</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ADH Group NYC | Home Improvement Company</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>adhnyc.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://www.adhnyc.com/hvac-installation-bronx-ny/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>infoes@adhnyc.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Bronx NY</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>76</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>heat pump installation Bronx NY</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-09 20:42 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-09.xlsx
+++ b/output/leads_2026-10-09.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1000,7 +1000,6 @@
           <t>infoes@adhnyc.com</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>Bronx NY</t>
@@ -1020,6 +1019,122 @@
         </is>
       </c>
       <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation in Carmel</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>triangleheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://www.triangleheatingandair.com/locations/carmel-in/heat-pump-installation</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>info@triangleheatingandair.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(833) 583-1095</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Carmel IN</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>90</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>heat pump installation Carmel IN</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Affordable Air and Plumbing</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>affordableairconditioningandheating.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://www.affordableairconditioningandheating.com/services/heating/furnaces</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>True Local</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>contact@affordableairandplumbing.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>239-772-0087</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Cape Coral FL</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>80</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>furnace repair Cape Coral FL</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-09 20:52 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-09.xlsx
+++ b/output/leads_2026-10-09.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1045,7 +1045,6 @@
           <t>https://www.triangleheatingandair.com/locations/carmel-in/heat-pump-installation</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>info@triangleheatingandair.com</t>
@@ -1135,6 +1134,66 @@
         </is>
       </c>
       <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>The Scoop</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>thescoop.guide</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://thescoop.guide/tx/odessa/hvac/furnace-heating/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Jeff Wilson</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>hello@thescoop.guide</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>(432) 552-8127</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Odessa TX</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>90</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>furnace repair Odessa TX</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-09 20:54 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-09.xlsx
+++ b/output/leads_2026-10-09.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1199,6 +1199,118 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Roof Replacement in Athens</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>georgiaroofreplacement.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://georgiaroofreplacement.com/locations/athens-ga/roof-replacement</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>info@georgiaroofreplacement.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>(229) 374-0018</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Athens GA</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>90</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>roof replacement Athens GA</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Professional Roofing Contractor | Lafayette, IN | ACPP Construction Services LLC</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>acppconstructionservices.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.acppconstructionservices.com/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>info@acppconstructionservices.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(765) 430-7510</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Lafayette IN</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>80</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>roofing contractor Lafayette IN</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>